<commit_message>
feat(be): update weekly evaluation AI logic, mock data seeding, and task import mapping
</commit_message>
<xml_diff>
--- a/templates/DataCrawler.xlsx
+++ b/templates/DataCrawler.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NodeJS\NexCampus\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NodeJS\NexCampus\NexCampus-BE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4407294-D294-476D-B192-C7E5845A3A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B3003FF-DC1B-4F39-9608-389A8706DBDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="330" windowWidth="29040" windowHeight="15990" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="308">
   <si>
     <t>KẾ HOẠCH PHÂN CÔNG TASK - DỰ ÁN CRAWL DATA</t>
   </si>
@@ -958,6 +958,9 @@
   </si>
   <si>
     <t>Phase</t>
+  </si>
+  <si>
+    <t>Email</t>
   </si>
 </sst>
 </file>
@@ -6145,19 +6148,19 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000000000000}">
           <x14:formula1>
-            <xm:f>Lists!$D$2:$D$5</xm:f>
+            <xm:f>Lists!$E$2:$E$5</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B46</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000002000000}">
           <x14:formula1>
-            <xm:f>Lists!$C$2:$C$4</xm:f>
+            <xm:f>Lists!$D$2:$D$4</xm:f>
           </x14:formula1>
           <xm:sqref>H2:H46</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" xr:uid="{00000000-0002-0000-0100-000003000000}">
           <x14:formula1>
-            <xm:f>Lists!$B$2:$B$6</xm:f>
+            <xm:f>Lists!$C$2:$C$6</xm:f>
           </x14:formula1>
           <xm:sqref>I2:I46</xm:sqref>
         </x14:dataValidation>
@@ -8357,28 +8360,30 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:M1000"/>
+  <dimension ref="A1:N1000"/>
   <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="20.8984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="25" width="8.59765625" customWidth="1"/>
+    <col min="1" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="20.8984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="26" width="8.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="13.8">
+    <row r="1" spans="1:14" ht="13.8">
       <c r="A1" s="1" t="s">
         <v>305</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>306</v>
       </c>
-      <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -8387,59 +8392,63 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="1:13" ht="13.8">
+    <row r="2" spans="1:14" ht="13.8">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="13.8">
+    <row r="3" spans="1:14" ht="13.8">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="13.8">
+    <row r="4" spans="1:14" ht="13.8">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="13.8">
-      <c r="B5" s="3" t="s">
+    <row r="5" spans="1:14" ht="13.8">
+      <c r="C5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="13.8">
-      <c r="B6" s="3" t="s">
+    <row r="6" spans="1:14" ht="13.8">
+      <c r="C6" s="3" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add DataCrawler template for initial data collection
</commit_message>
<xml_diff>
--- a/templates/DataCrawler.xlsx
+++ b/templates/DataCrawler.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NodeJS\NexCampus\NexCampus-BE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B3003FF-DC1B-4F39-9608-389A8706DBDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92E92B2E-13FD-4336-BF95-D3BC8817EEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="330" windowWidth="29040" windowHeight="15990" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="330" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -3163,10 +3163,10 @@
         <v>8</v>
       </c>
       <c r="J2" s="5">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="K2" s="5">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="L2" s="6">
         <v>1</v>
@@ -3206,10 +3206,10 @@
         <v>8</v>
       </c>
       <c r="J3" s="5">
-        <v>46204</v>
+        <v>46235</v>
       </c>
       <c r="K3" s="5">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="L3" s="6">
         <v>1</v>
@@ -3251,10 +3251,10 @@
         <v>8</v>
       </c>
       <c r="J4" s="5">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="K4" s="5">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="L4" s="6">
         <v>1.5</v>
@@ -3296,10 +3296,10 @@
         <v>8</v>
       </c>
       <c r="J5" s="5">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="K5" s="5">
-        <v>46206</v>
+        <v>46238</v>
       </c>
       <c r="L5" s="6">
         <v>0.5</v>
@@ -3341,10 +3341,10 @@
         <v>8</v>
       </c>
       <c r="J6" s="5">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="K6" s="5">
-        <v>46207</v>
+        <v>46238</v>
       </c>
       <c r="L6" s="6">
         <v>0.5</v>
@@ -3386,10 +3386,10 @@
         <v>8</v>
       </c>
       <c r="J7" s="5">
-        <v>46207</v>
+        <v>46238</v>
       </c>
       <c r="K7" s="5">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="L7" s="6">
         <v>1</v>
@@ -3431,10 +3431,10 @@
         <v>8</v>
       </c>
       <c r="J8" s="5">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="K8" s="5">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="L8" s="6">
         <v>1</v>
@@ -3476,10 +3476,10 @@
         <v>8</v>
       </c>
       <c r="J9" s="5">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="K9" s="5">
-        <v>46207</v>
+        <v>46238</v>
       </c>
       <c r="L9" s="6">
         <v>1</v>
@@ -3521,10 +3521,10 @@
         <v>8</v>
       </c>
       <c r="J10" s="5">
-        <v>46207</v>
+        <v>46238</v>
       </c>
       <c r="K10" s="5">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="L10" s="6">
         <v>1</v>
@@ -3566,10 +3566,10 @@
         <v>8</v>
       </c>
       <c r="J11" s="5">
-        <v>46205</v>
+        <v>46236</v>
       </c>
       <c r="K11" s="5">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="L11" s="6">
         <v>0.5</v>
@@ -3611,10 +3611,10 @@
         <v>8</v>
       </c>
       <c r="J12" s="5">
-        <v>46206</v>
+        <v>46237</v>
       </c>
       <c r="K12" s="5">
-        <v>46207</v>
+        <v>46238</v>
       </c>
       <c r="L12" s="6">
         <v>1</v>
@@ -3656,10 +3656,10 @@
         <v>8</v>
       </c>
       <c r="J13" s="5">
-        <v>46207</v>
+        <v>46238</v>
       </c>
       <c r="K13" s="5">
-        <v>46208</v>
+        <v>46239</v>
       </c>
       <c r="L13" s="6">
         <v>1</v>
@@ -3701,10 +3701,10 @@
         <v>8</v>
       </c>
       <c r="J14" s="5">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="K14" s="5">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="L14" s="6">
         <v>1.5</v>
@@ -3746,10 +3746,10 @@
         <v>8</v>
       </c>
       <c r="J15" s="5">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="K15" s="5">
-        <v>46211</v>
+        <v>46242</v>
       </c>
       <c r="L15" s="6">
         <v>1</v>
@@ -3791,10 +3791,10 @@
         <v>8</v>
       </c>
       <c r="J16" s="5">
-        <v>46211</v>
+        <v>46242</v>
       </c>
       <c r="K16" s="5">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="L16" s="6">
         <v>1.5</v>
@@ -3836,10 +3836,10 @@
         <v>8</v>
       </c>
       <c r="J17" s="5">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="K17" s="5">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="L17" s="6">
         <v>1</v>
@@ -3881,10 +3881,10 @@
         <v>8</v>
       </c>
       <c r="J18" s="5">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="K18" s="5">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="L18" s="6">
         <v>0.75</v>
@@ -3926,10 +3926,10 @@
         <v>8</v>
       </c>
       <c r="J19" s="5">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="K19" s="5">
-        <v>46211</v>
+        <v>46242</v>
       </c>
       <c r="L19" s="6">
         <v>2</v>
@@ -3971,10 +3971,10 @@
         <v>8</v>
       </c>
       <c r="J20" s="5">
-        <v>46211</v>
+        <v>46242</v>
       </c>
       <c r="K20" s="5">
-        <v>46213</v>
+        <v>46244</v>
       </c>
       <c r="L20" s="6">
         <v>2</v>
@@ -4016,10 +4016,10 @@
         <v>8</v>
       </c>
       <c r="J21" s="5">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="K21" s="5">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="L21" s="6">
         <v>1</v>
@@ -4061,10 +4061,10 @@
         <v>8</v>
       </c>
       <c r="J22" s="5">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="K22" s="5">
-        <v>46215</v>
+        <v>46246</v>
       </c>
       <c r="L22" s="6">
         <v>1</v>
@@ -4106,10 +4106,10 @@
         <v>8</v>
       </c>
       <c r="J23" s="5">
-        <v>46209</v>
+        <v>46240</v>
       </c>
       <c r="K23" s="5">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="L23" s="6">
         <v>1</v>
@@ -4151,10 +4151,10 @@
         <v>8</v>
       </c>
       <c r="J24" s="5">
-        <v>46210</v>
+        <v>46241</v>
       </c>
       <c r="K24" s="5">
-        <v>46211</v>
+        <v>46242</v>
       </c>
       <c r="L24" s="6">
         <v>1</v>
@@ -4196,10 +4196,10 @@
         <v>8</v>
       </c>
       <c r="J25" s="5">
-        <v>46211</v>
+        <v>46242</v>
       </c>
       <c r="K25" s="5">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="L25" s="6">
         <v>1</v>
@@ -4241,10 +4241,10 @@
         <v>8</v>
       </c>
       <c r="J26" s="5">
-        <v>46212</v>
+        <v>46243</v>
       </c>
       <c r="K26" s="5">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="L26" s="6">
         <v>1.5</v>
@@ -4286,10 +4286,10 @@
         <v>8</v>
       </c>
       <c r="J27" s="5">
-        <v>46214</v>
+        <v>46245</v>
       </c>
       <c r="K27" s="5">
-        <v>46215</v>
+        <v>46246</v>
       </c>
       <c r="L27" s="6">
         <v>1</v>
@@ -4331,10 +4331,10 @@
         <v>8</v>
       </c>
       <c r="J28" s="5">
-        <v>46216</v>
+        <v>46247</v>
       </c>
       <c r="K28" s="5">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="L28" s="6">
         <v>1.5</v>
@@ -4376,10 +4376,10 @@
         <v>8</v>
       </c>
       <c r="J29" s="5">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="K29" s="5">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="L29" s="6">
         <v>1</v>
@@ -4421,10 +4421,10 @@
         <v>8</v>
       </c>
       <c r="J30" s="5">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="K30" s="5">
-        <v>46220</v>
+        <v>46251</v>
       </c>
       <c r="L30" s="6">
         <v>1</v>
@@ -4466,10 +4466,10 @@
         <v>8</v>
       </c>
       <c r="J31" s="5">
-        <v>46216</v>
+        <v>46247</v>
       </c>
       <c r="K31" s="5">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="L31" s="6">
         <v>1.5</v>
@@ -4511,10 +4511,10 @@
         <v>8</v>
       </c>
       <c r="J32" s="5">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="K32" s="5">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="L32" s="6">
         <v>1</v>
@@ -4556,10 +4556,10 @@
         <v>8</v>
       </c>
       <c r="J33" s="5">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="K33" s="5">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="L33" s="6">
         <v>1.5</v>
@@ -4601,10 +4601,10 @@
         <v>8</v>
       </c>
       <c r="J34" s="5">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="K34" s="5">
-        <v>46222</v>
+        <v>46253</v>
       </c>
       <c r="L34" s="6">
         <v>1</v>
@@ -4646,10 +4646,10 @@
         <v>8</v>
       </c>
       <c r="J35" s="5">
-        <v>46216</v>
+        <v>46247</v>
       </c>
       <c r="K35" s="5">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="L35" s="6">
         <v>1.5</v>
@@ -4691,10 +4691,10 @@
         <v>8</v>
       </c>
       <c r="J36" s="5">
-        <v>46218</v>
+        <v>46249</v>
       </c>
       <c r="K36" s="5">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="L36" s="6">
         <v>1</v>
@@ -4736,10 +4736,10 @@
         <v>8</v>
       </c>
       <c r="J37" s="5">
-        <v>46219</v>
+        <v>46250</v>
       </c>
       <c r="K37" s="5">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="L37" s="6">
         <v>1.5</v>
@@ -4781,10 +4781,10 @@
         <v>8</v>
       </c>
       <c r="J38" s="5">
-        <v>46221</v>
+        <v>46252</v>
       </c>
       <c r="K38" s="5">
-        <v>46222</v>
+        <v>46253</v>
       </c>
       <c r="L38" s="6">
         <v>1</v>
@@ -4826,10 +4826,10 @@
         <v>8</v>
       </c>
       <c r="J39" s="5">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="K39" s="5">
-        <v>46224</v>
+        <v>46255</v>
       </c>
       <c r="L39" s="6">
         <v>1</v>
@@ -4871,10 +4871,10 @@
         <v>8</v>
       </c>
       <c r="J40" s="5">
-        <v>46224</v>
+        <v>46255</v>
       </c>
       <c r="K40" s="5">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="L40" s="6">
         <v>1.5</v>
@@ -4916,10 +4916,10 @@
         <v>8</v>
       </c>
       <c r="J41" s="5">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="K41" s="5">
-        <v>46224</v>
+        <v>46255</v>
       </c>
       <c r="L41" s="6">
         <v>1</v>
@@ -4961,10 +4961,10 @@
         <v>8</v>
       </c>
       <c r="J42" s="5">
-        <v>46224</v>
+        <v>46255</v>
       </c>
       <c r="K42" s="5">
-        <v>46225</v>
+        <v>46256</v>
       </c>
       <c r="L42" s="6">
         <v>1</v>
@@ -5006,10 +5006,10 @@
         <v>8</v>
       </c>
       <c r="J43" s="5">
-        <v>46225</v>
+        <v>46256</v>
       </c>
       <c r="K43" s="5">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="L43" s="6">
         <v>1.5</v>
@@ -5051,10 +5051,10 @@
         <v>8</v>
       </c>
       <c r="J44" s="5">
-        <v>46223</v>
+        <v>46254</v>
       </c>
       <c r="K44" s="5">
-        <v>46224</v>
+        <v>46255</v>
       </c>
       <c r="L44" s="6">
         <v>0.75</v>
@@ -5094,10 +5094,10 @@
         <v>8</v>
       </c>
       <c r="J45" s="5">
-        <v>46224</v>
+        <v>46255</v>
       </c>
       <c r="K45" s="5">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="L45" s="6">
         <v>1</v>
@@ -5139,10 +5139,10 @@
         <v>8</v>
       </c>
       <c r="J46" s="5">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="K46" s="5">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="L46" s="6">
         <v>1.5</v>

</xml_diff>

<commit_message>
feat(task-assignment): add email lookup and direct assign/unassign task APIs
</commit_message>
<xml_diff>
--- a/templates/DataCrawler.xlsx
+++ b/templates/DataCrawler.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NodeJS\NexCampus\NexCampus-BE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92E92B2E-13FD-4336-BF95-D3BC8817EEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF20DC41-6ABB-4894-98F2-0BE349B4F254}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="330" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32370" yWindow="4020" windowWidth="21600" windowHeight="11430" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="F5" s="3">
         <f>COUNTIF(Task_Phan_Cong!I2:I46,"To Do")</f>
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="13.8">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="F6" s="3">
         <f>COUNTIF(Task_Phan_Cong!I2:I46,"In Progress")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="13.8">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="F7" s="3">
         <f>COUNTIF(Task_Phan_Cong!I2:I46,"Review")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="13.8">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="F8" s="3">
         <f>COUNTIF(Task_Phan_Cong!I2:I46,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="13.8">
@@ -5048,7 +5048,7 @@
         <v>18</v>
       </c>
       <c r="I44" s="4" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="J44" s="5">
         <v>46254</v>
@@ -5091,7 +5091,7 @@
         <v>18</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="J45" s="5">
         <v>46255</v>
@@ -5136,7 +5136,7 @@
         <v>18</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="J46" s="5">
         <v>46257</v>

</xml_diff>